<commit_message>
Add matrix-driven E2E coverage for applications, clients, policies, and create-application flows Expand the capability framework with persona-specific dashboard, list, and detail tests; add Excel-driven create-application workflows (TMD, validation, document upload); include CI matrix workflow and updated matrix generator.
</commit_message>
<xml_diff>
--- a/projects/keyinvest/data/matrix.xlsx
+++ b/projects/keyinvest/data/matrix.xlsx
@@ -4,6 +4,8 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="TestMatrix" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateApplicationData" sheetId="2" r:id="rId2"/>
+    <sheet name="CreateApplicationValidation" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +399,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:K31"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" customWidth="1"/>
+    <col min="18" max="18" width="16.6640625" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" customWidth="1"/>
+    <col min="20" max="20" width="16.6640625" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
+    <col min="24" max="24" width="16.6640625" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +451,18 @@
       <c r="G1" t="str">
         <v>expectedResult</v>
       </c>
+      <c r="H1" t="str">
+        <v>bondType</v>
+      </c>
+      <c r="I1" t="str">
+        <v>dataRow</v>
+      </c>
+      <c r="J1" t="str">
+        <v>scenario</v>
+      </c>
+      <c r="K1" t="str">
+        <v>documentSet</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -435,12 +477,6 @@
       <c r="D2" t="str">
         <v>guest</v>
       </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
       <c r="G2" t="str">
         <v>success</v>
       </c>
@@ -458,12 +494,6 @@
       <c r="D3" t="str">
         <v>investor</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
       <c r="G3" t="str">
         <v>success</v>
       </c>
@@ -481,12 +511,6 @@
       <c r="D4" t="str">
         <v>funeral</v>
       </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
       <c r="G4" t="str">
         <v>success</v>
       </c>
@@ -504,12 +528,6 @@
       <c r="D5" t="str">
         <v>adviser</v>
       </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
       <c r="G5" t="str">
         <v>success</v>
       </c>
@@ -527,12 +545,6 @@
       <c r="D6" t="str">
         <v>admin</v>
       </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
       <c r="G6" t="str">
         <v>success</v>
       </c>
@@ -568,19 +580,19 @@
         <v>Y</v>
       </c>
       <c r="C8" t="str">
-        <v>dashboard</v>
+        <v>login</v>
       </c>
       <c r="D8" t="str">
-        <v>investor</v>
+        <v>adviser</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>baduser</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>WrongPass123</v>
       </c>
       <c r="G8" t="str">
-        <v>success</v>
+        <v>validation_error</v>
       </c>
     </row>
     <row r="9">
@@ -591,16 +603,10 @@
         <v>Y</v>
       </c>
       <c r="C9" t="str">
-        <v>dashboard</v>
+        <v>dashboard-full</v>
       </c>
       <c r="D9" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v/>
+        <v>investor</v>
       </c>
       <c r="G9" t="str">
         <v>success</v>
@@ -614,16 +620,10 @@
         <v>Y</v>
       </c>
       <c r="C10" t="str">
-        <v>dashboard</v>
+        <v>dashboard-full</v>
       </c>
       <c r="D10" t="str">
-        <v>adviser</v>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
+        <v>funeral</v>
       </c>
       <c r="G10" t="str">
         <v>success</v>
@@ -637,16 +637,10 @@
         <v>Y</v>
       </c>
       <c r="C11" t="str">
-        <v>dashboard</v>
+        <v>dashboard-full</v>
       </c>
       <c r="D11" t="str">
-        <v>admin</v>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v/>
+        <v>adviser</v>
       </c>
       <c r="G11" t="str">
         <v>success</v>
@@ -660,16 +654,10 @@
         <v>Y</v>
       </c>
       <c r="C12" t="str">
-        <v>dashboard-links</v>
+        <v>dashboard-full</v>
       </c>
       <c r="D12" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
-        <v/>
+        <v>admin</v>
       </c>
       <c r="G12" t="str">
         <v>success</v>
@@ -683,16 +671,10 @@
         <v>Y</v>
       </c>
       <c r="C13" t="str">
-        <v>dashboard-exports</v>
+        <v>clients-full</v>
       </c>
       <c r="D13" t="str">
         <v>funeral</v>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v/>
       </c>
       <c r="G13" t="str">
         <v>success</v>
@@ -706,16 +688,10 @@
         <v>Y</v>
       </c>
       <c r="C14" t="str">
-        <v>dashboard-exports</v>
+        <v>clients-full</v>
       </c>
       <c r="D14" t="str">
         <v>adviser</v>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v/>
       </c>
       <c r="G14" t="str">
         <v>success</v>
@@ -729,16 +705,10 @@
         <v>Y</v>
       </c>
       <c r="C15" t="str">
-        <v>portfolio-check</v>
+        <v>clients-full</v>
       </c>
       <c r="D15" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
-        <v/>
+        <v>investor</v>
       </c>
       <c r="G15" t="str">
         <v>success</v>
@@ -752,16 +722,10 @@
         <v>Y</v>
       </c>
       <c r="C16" t="str">
-        <v>portfolio-check</v>
+        <v>policies-full</v>
       </c>
       <c r="D16" t="str">
-        <v>adviser</v>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v/>
+        <v>funeral</v>
       </c>
       <c r="G16" t="str">
         <v>success</v>
@@ -775,16 +739,10 @@
         <v>Y</v>
       </c>
       <c r="C17" t="str">
-        <v>recent-app</v>
+        <v>policies-full</v>
       </c>
       <c r="D17" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v/>
+        <v>adviser</v>
       </c>
       <c r="G17" t="str">
         <v>success</v>
@@ -798,16 +756,10 @@
         <v>Y</v>
       </c>
       <c r="C18" t="str">
-        <v>recent-app</v>
+        <v>policies-full</v>
       </c>
       <c r="D18" t="str">
-        <v>adviser</v>
-      </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-      <c r="F18" t="str">
-        <v/>
+        <v>investor</v>
       </c>
       <c r="G18" t="str">
         <v>success</v>
@@ -821,16 +773,10 @@
         <v>Y</v>
       </c>
       <c r="C19" t="str">
-        <v>summary-filters</v>
+        <v>policies-full</v>
       </c>
       <c r="D19" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E19" t="str">
-        <v/>
-      </c>
-      <c r="F19" t="str">
-        <v/>
+        <v>admin</v>
       </c>
       <c r="G19" t="str">
         <v>success</v>
@@ -844,16 +790,10 @@
         <v>Y</v>
       </c>
       <c r="C20" t="str">
-        <v>summary-filters</v>
+        <v>applications-full</v>
       </c>
       <c r="D20" t="str">
-        <v>adviser</v>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
-        <v/>
+        <v>funeral</v>
       </c>
       <c r="G20" t="str">
         <v>success</v>
@@ -867,16 +807,10 @@
         <v>Y</v>
       </c>
       <c r="C21" t="str">
-        <v>dashboard-full</v>
+        <v>applications-full</v>
       </c>
       <c r="D21" t="str">
-        <v>funeral</v>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v/>
+        <v>adviser</v>
       </c>
       <c r="G21" t="str">
         <v>success</v>
@@ -890,16 +824,10 @@
         <v>Y</v>
       </c>
       <c r="C22" t="str">
-        <v>dashboard-full</v>
+        <v>applications-full</v>
       </c>
       <c r="D22" t="str">
-        <v>adviser</v>
-      </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
-        <v/>
+        <v>investor</v>
       </c>
       <c r="G22" t="str">
         <v>success</v>
@@ -913,24 +841,817 @@
         <v>Y</v>
       </c>
       <c r="C23" t="str">
-        <v>funeral-full</v>
+        <v>applications-full</v>
       </c>
       <c r="D23" t="str">
+        <v>admin</v>
+      </c>
+      <c r="G23" t="str">
+        <v>success</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC-23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>N</v>
+      </c>
+      <c r="C24" t="str">
+        <v>create-application-full</v>
+      </c>
+      <c r="D24" t="str">
         <v>funeral</v>
       </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-      <c r="F23" t="str">
-        <v/>
-      </c>
-      <c r="G23" t="str">
-        <v>success</v>
+      <c r="G24" t="str">
+        <v>success</v>
+      </c>
+      <c r="H24" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="I24" t="str">
+        <v>PREPAID-FUNERAL-01</v>
+      </c>
+      <c r="K24" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC-24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>N</v>
+      </c>
+      <c r="C25" t="str">
+        <v>create-application-full</v>
+      </c>
+      <c r="D25" t="str">
+        <v>funeral</v>
+      </c>
+      <c r="G25" t="str">
+        <v>success</v>
+      </c>
+      <c r="H25" t="str">
+        <v>NOMINATED</v>
+      </c>
+      <c r="I25" t="str">
+        <v>NOMINATED-FUNERAL-01</v>
+      </c>
+      <c r="K25" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC-25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C26" t="str">
+        <v>create-application-full</v>
+      </c>
+      <c r="D26" t="str">
+        <v>adviser</v>
+      </c>
+      <c r="G26" t="str">
+        <v>success</v>
+      </c>
+      <c r="H26" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="I26" t="str">
+        <v>PREPAID-ADVISER-01</v>
+      </c>
+      <c r="K26" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC-26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C27" t="str">
+        <v>create-application-full</v>
+      </c>
+      <c r="D27" t="str">
+        <v>investor</v>
+      </c>
+      <c r="G27" t="str">
+        <v>success</v>
+      </c>
+      <c r="H27" t="str">
+        <v>NOMINATED</v>
+      </c>
+      <c r="I27" t="str">
+        <v>NOMINATED-INVESTOR-01</v>
+      </c>
+      <c r="K27" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC-27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C28" t="str">
+        <v>create-application-full</v>
+      </c>
+      <c r="D28" t="str">
+        <v>guest</v>
+      </c>
+      <c r="G28" t="str">
+        <v>success</v>
+      </c>
+      <c r="H28" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="I28" t="str">
+        <v>PREPAID-GUEST-01</v>
+      </c>
+      <c r="K28" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC-28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C29" t="str">
+        <v>create-application-tmd</v>
+      </c>
+      <c r="D29" t="str">
+        <v>funeral</v>
+      </c>
+      <c r="G29" t="str">
+        <v>success</v>
+      </c>
+      <c r="J29" t="str">
+        <v>tmd-suite</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC-29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C30" t="str">
+        <v>create-application-tmd</v>
+      </c>
+      <c r="D30" t="str">
+        <v>adviser</v>
+      </c>
+      <c r="G30" t="str">
+        <v>success</v>
+      </c>
+      <c r="J30" t="str">
+        <v>tmd-suite</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC-30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C31" t="str">
+        <v>create-application-validation</v>
+      </c>
+      <c r="D31" t="str">
+        <v>funeral</v>
+      </c>
+      <c r="G31" t="str">
+        <v>validation_error</v>
+      </c>
+      <c r="J31" t="str">
+        <v>tmd-wrong-q1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U6"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" customWidth="1"/>
+    <col min="18" max="18" width="16.6640625" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" customWidth="1"/>
+    <col min="20" max="20" width="16.6640625" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
+    <col min="24" max="24" width="16.6640625" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>dataRow</v>
+      </c>
+      <c r="B1" t="str">
+        <v>bondType</v>
+      </c>
+      <c r="C1" t="str">
+        <v>tmdAnswers</v>
+      </c>
+      <c r="D1" t="str">
+        <v>title</v>
+      </c>
+      <c r="E1" t="str">
+        <v>givenName</v>
+      </c>
+      <c r="F1" t="str">
+        <v>surname</v>
+      </c>
+      <c r="G1" t="str">
+        <v>email</v>
+      </c>
+      <c r="H1" t="str">
+        <v>dob</v>
+      </c>
+      <c r="I1" t="str">
+        <v>gender</v>
+      </c>
+      <c r="J1" t="str">
+        <v>phone</v>
+      </c>
+      <c r="K1" t="str">
+        <v>streetNumber</v>
+      </c>
+      <c r="L1" t="str">
+        <v>streetName</v>
+      </c>
+      <c r="M1" t="str">
+        <v>streetType</v>
+      </c>
+      <c r="N1" t="str">
+        <v>suburb</v>
+      </c>
+      <c r="O1" t="str">
+        <v>state</v>
+      </c>
+      <c r="P1" t="str">
+        <v>postcode</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>country</v>
+      </c>
+      <c r="R1" t="str">
+        <v>initialAmount</v>
+      </c>
+      <c r="S1" t="str">
+        <v>defaultCapital</v>
+      </c>
+      <c r="T1" t="str">
+        <v>paymentType</v>
+      </c>
+      <c r="U1" t="str">
+        <v>documentSet</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PREPAID-FUNERAL-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C2" t="str">
+        <v>yes,no,no,no</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Playwright</v>
+      </c>
+      <c r="F2" t="str">
+        <v>FuneralPrepaid</v>
+      </c>
+      <c r="G2" t="str">
+        <v>shivprasad.mane@evoltech.com.au</v>
+      </c>
+      <c r="H2" t="str">
+        <v>1980-01-15</v>
+      </c>
+      <c r="I2" t="str">
+        <v>male</v>
+      </c>
+      <c r="J2" t="str">
+        <v>0412345678</v>
+      </c>
+      <c r="K2" t="str">
+        <v>10</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Main</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Street</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Sydney</v>
+      </c>
+      <c r="O2" t="str">
+        <v>New South Wales</v>
+      </c>
+      <c r="P2" t="str">
+        <v>2000</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="R2" t="str">
+        <v>1000</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="T2" t="str">
+        <v>BPAY</v>
+      </c>
+      <c r="U2" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>NOMINATED-FUNERAL-01</v>
+      </c>
+      <c r="B3" t="str">
+        <v>NOMINATED</v>
+      </c>
+      <c r="C3" t="str">
+        <v>yes,no,no,no</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ms</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Playwright</v>
+      </c>
+      <c r="F3" t="str">
+        <v>FuneralNominated</v>
+      </c>
+      <c r="G3" t="str">
+        <v>shivprasad.mane@evoltech.com.au</v>
+      </c>
+      <c r="H3" t="str">
+        <v>1975-06-20</v>
+      </c>
+      <c r="I3" t="str">
+        <v>female</v>
+      </c>
+      <c r="J3" t="str">
+        <v>0412345679</v>
+      </c>
+      <c r="K3" t="str">
+        <v>20</v>
+      </c>
+      <c r="L3" t="str">
+        <v>George</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Street</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Victoria</v>
+      </c>
+      <c r="P3" t="str">
+        <v>3000</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="R3" t="str">
+        <v>1500</v>
+      </c>
+      <c r="S3" t="str">
+        <v>N</v>
+      </c>
+      <c r="T3" t="str">
+        <v>BPAY</v>
+      </c>
+      <c r="U3" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PREPAID-ADVISER-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C4" t="str">
+        <v>yes,no,no,no</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Playwright</v>
+      </c>
+      <c r="F4" t="str">
+        <v>AdviserPrepaid</v>
+      </c>
+      <c r="G4" t="str">
+        <v>shivprasad.mane@evoltech.com.au</v>
+      </c>
+      <c r="H4" t="str">
+        <v>1982-03-10</v>
+      </c>
+      <c r="I4" t="str">
+        <v>male</v>
+      </c>
+      <c r="J4" t="str">
+        <v>0412345680</v>
+      </c>
+      <c r="K4" t="str">
+        <v>5</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Collins</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Street</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Melbourne</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Victoria</v>
+      </c>
+      <c r="P4" t="str">
+        <v>3000</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="R4" t="str">
+        <v>1000</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="T4" t="str">
+        <v>BPAY</v>
+      </c>
+      <c r="U4" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>NOMINATED-INVESTOR-01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>NOMINATED</v>
+      </c>
+      <c r="C5" t="str">
+        <v>yes,no,no,no</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Playwright</v>
+      </c>
+      <c r="F5" t="str">
+        <v>InvestorNominated</v>
+      </c>
+      <c r="G5" t="str">
+        <v>shivprasad.mane@evoltech.com.au</v>
+      </c>
+      <c r="H5" t="str">
+        <v>1978-11-05</v>
+      </c>
+      <c r="I5" t="str">
+        <v>male</v>
+      </c>
+      <c r="J5" t="str">
+        <v>0412345681</v>
+      </c>
+      <c r="K5" t="str">
+        <v>8</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Queen</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Street</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Brisbane</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Queensland</v>
+      </c>
+      <c r="P5" t="str">
+        <v>4000</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="R5" t="str">
+        <v>1200</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Y</v>
+      </c>
+      <c r="T5" t="str">
+        <v>BPAY</v>
+      </c>
+      <c r="U5" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PREPAID-GUEST-01</v>
+      </c>
+      <c r="B6" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C6" t="str">
+        <v>yes,no,no,no</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Playwright</v>
+      </c>
+      <c r="F6" t="str">
+        <v>GuestPrepaid</v>
+      </c>
+      <c r="G6" t="str">
+        <v>shivprasad.mane@evoltech.com.au</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1990-07-22</v>
+      </c>
+      <c r="I6" t="str">
+        <v>male</v>
+      </c>
+      <c r="J6" t="str">
+        <v>0412345682</v>
+      </c>
+      <c r="K6" t="str">
+        <v>12</v>
+      </c>
+      <c r="L6" t="str">
+        <v>King</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Street</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Perth</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Western Australia</v>
+      </c>
+      <c r="P6" t="str">
+        <v>6000</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Australia</v>
+      </c>
+      <c r="R6" t="str">
+        <v>1000</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="T6" t="str">
+        <v>BPAY</v>
+      </c>
+      <c r="U6" t="str">
+        <v>default-docs</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:U6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H6"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" customWidth="1"/>
+    <col min="18" max="18" width="16.6640625" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" customWidth="1"/>
+    <col min="20" max="20" width="16.6640625" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
+    <col min="24" max="24" width="16.6640625" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>scenarioId</v>
+      </c>
+      <c r="B1" t="str">
+        <v>bondType</v>
+      </c>
+      <c r="C1" t="str">
+        <v>step</v>
+      </c>
+      <c r="D1" t="str">
+        <v>testCase</v>
+      </c>
+      <c r="E1" t="str">
+        <v>field</v>
+      </c>
+      <c r="F1" t="str">
+        <v>inputValue</v>
+      </c>
+      <c r="G1" t="str">
+        <v>expectedError</v>
+      </c>
+      <c r="H1" t="str">
+        <v>persona</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>tmd-wrong-q1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C2" t="str">
+        <v>0</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TMD wrong answer</v>
+      </c>
+      <c r="E2" t="str">
+        <v>tmdQ1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>no</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Warning visible, Confirm disabled</v>
+      </c>
+      <c r="H2" t="str">
+        <v>funeral</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>tmd-no-bond</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C3" t="str">
+        <v>0</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TMD no bond</v>
+      </c>
+      <c r="E3" t="str">
+        <v>bondType</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Confirm disabled</v>
+      </c>
+      <c r="H3" t="str">
+        <v>funeral</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>tmd-api-match</v>
+      </c>
+      <c r="B4" t="str">
+        <v>NOMINATED</v>
+      </c>
+      <c r="C4" t="str">
+        <v>0</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TMD API load</v>
+      </c>
+      <c r="G4" t="str">
+        <v>all API questions visible</v>
+      </c>
+      <c r="H4" t="str">
+        <v>funeral</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>tmd-suite</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C5" t="str">
+        <v>0</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TMD API load</v>
+      </c>
+      <c r="G5" t="str">
+        <v>all API questions visible</v>
+      </c>
+      <c r="H5" t="str">
+        <v>funeral</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>step1-invalid-email</v>
+      </c>
+      <c r="B6" t="str">
+        <v>PREPAID</v>
+      </c>
+      <c r="C6" t="str">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Email format</v>
+      </c>
+      <c r="E6" t="str">
+        <v>email</v>
+      </c>
+      <c r="F6" t="str">
+        <v>not-an-email</v>
+      </c>
+      <c r="G6" t="str">
+        <v>invalid email</v>
+      </c>
+      <c r="H6" t="str">
+        <v>funeral</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>